<commit_message>
updated the model to account for visualization block order, Tukey adjustment, sensitivity analysis
</commit_message>
<xml_diff>
--- a/Subjective Feedback_Design Domain Experts.xlsx
+++ b/Subjective Feedback_Design Domain Experts.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B4F365FD-FC1B-4D96-BE6E-BDD0E35F10D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2547985456586/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{B4F365FD-FC1B-4D96-BE6E-BDD0E35F10D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF928DEF-A358-354E-95FF-F976ACA2BDE4}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30980" yWindow="2340" windowWidth="37060" windowHeight="26340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,9 +62,6 @@
     <t>Select Excerpt / Quotes</t>
   </si>
   <si>
-    <t>P1</t>
-  </si>
-  <si>
     <t>Industrial Design</t>
   </si>
   <si>
@@ -71,6 +73,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>“I do like the whole pair design balance for where you have one thing in, one thing out. The radial one</t>
     </r>
@@ -80,6 +83,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Grouped Radial Chart)</t>
     </r>
@@ -88,6 +92,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> is a bit too complex to quickly read in that sense.”
 “But in the glyph even for like Timor-Leste and Brunei, countries that don't have a clean even data or like, they don't have a lot of import and exports, but it still doesn't look bad when not fully populated.”
@@ -99,6 +104,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Blossom Glyph)</t>
     </r>
@@ -107,19 +113,18 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> kinda makes a flower in the middle negative space too. I think that's fun.”</t>
     </r>
   </si>
   <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>“It's</t>
     </r>
@@ -129,6 +134,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(Blossom Glyph) </t>
     </r>
@@ -137,6 +143,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">like more soft and natural looking, like it feel less technical and more like a icon.” 
 “I mean, yeah, the the visual appearance is not separate from the information part.” </t>
@@ -147,6 +154,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(About Blossom Glyph)</t>
     </r>
@@ -155,14 +163,12 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
   </si>
   <si>
-    <t>P3</t>
-  </si>
-  <si>
     <t>Interaction Design</t>
   </si>
   <si>
@@ -174,6 +180,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>“I think my least favorite of the three is the radial chart</t>
     </r>
@@ -183,6 +190,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Grouped Radial Chart)</t>
     </r>
@@ -191,6 +199,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>. It's just it would take me a little longer, I think. I know it's the same stats, but I just feel like there's a lot more information to digest here.”
 “I'm surprised. I think the bar chart</t>
@@ -201,6 +210,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Diverging Bar Chart)</t>
     </r>
@@ -209,14 +219,12 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> was the best one alone, but I kind of don't like how the multiple bars look close together on the map.”</t>
     </r>
   </si>
   <si>
-    <t>P4</t>
-  </si>
-  <si>
     <t>Visual Communication Design</t>
   </si>
   <si>
@@ -225,6 +233,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>“I feel like this one</t>
     </r>
@@ -234,6 +243,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(Blossom Glyph) </t>
     </r>
@@ -242,6 +252,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>is more easy on the eyes.”
 “I think it's</t>
@@ -252,6 +263,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Blossom Glyph)</t>
     </r>
@@ -260,6 +272,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> the one that feels like it has a visual identity. The bar chart is maybe clearer, but it feels like a default chart. The glyph</t>
     </r>
@@ -269,6 +282,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Blossom Glyph)</t>
     </r>
@@ -277,6 +291,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> is like a visual form, not just a chart. It's nice that it's recognizable like that.”
 “But I would also say the aesthetics depend a lot on spacing, labels, or amount of color. Like if it's</t>
@@ -287,6 +302,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(attributes)</t>
     </r>
@@ -295,6 +311,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> meant to be more than 6 or 7. If those are handled well, it feels readable. If not, it could become pretty dense quickly.” </t>
     </r>
@@ -304,19 +321,18 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(About Blossom Glyph) </t>
     </r>
   </si>
   <si>
-    <t>P5</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>“In the radial chart</t>
     </r>
@@ -326,6 +342,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Grouped Radial Chart)</t>
     </r>
@@ -334,17 +351,33 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> I feel like the angle division are throwing me off. It's almost like it has to be a circle, but because of the groups, it's not. I wonder what that will look like with more than 5 groups, it maybe more hard to read.”
 “The left and right bars are just cleaner, easy for me to read.”</t>
     </r>
+  </si>
+  <si>
+    <t>E1</t>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>E3</t>
+  </si>
+  <si>
+    <t>E4</t>
+  </si>
+  <si>
+    <t>E5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -356,12 +389,14 @@
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -369,6 +404,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -376,6 +412,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -383,35 +420,41 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -494,19 +537,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -727,24 +770,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Z9"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="1"/>
-    <col min="2" max="2" width="25.42578125" customWidth="1"/>
-    <col min="3" max="4" width="20.5703125" customWidth="1"/>
-    <col min="5" max="5" width="25.7109375" customWidth="1"/>
-    <col min="6" max="6" width="55.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
+    <col min="3" max="4" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" customWidth="1"/>
+    <col min="6" max="6" width="55.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="39.75" customHeight="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -766,15 +809,15 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="38.25" customHeight="1">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:26" ht="38.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -796,15 +839,15 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="9.75" customHeight="1">
-      <c r="A3" s="12"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
+    <row r="3" spans="1:26" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="14"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
     </row>
-    <row r="4" spans="1:26" ht="45.75" customHeight="1">
+    <row r="4" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -824,12 +867,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="130.5">
+    <row r="5" spans="1:26" ht="140" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>9</v>
       </c>
       <c r="C5" s="4">
         <v>4</v>
@@ -838,18 +881,18 @@
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="6" spans="1:26" ht="60">
+    <row r="6" spans="1:26" ht="70" x14ac:dyDescent="0.15">
       <c r="A6" s="6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="7">
         <v>8</v>
@@ -858,10 +901,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
@@ -884,12 +927,12 @@
       <c r="Y6" s="9"/>
       <c r="Z6" s="9"/>
     </row>
-    <row r="7" spans="1:26" ht="96">
+    <row r="7" spans="1:26" ht="112" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C7" s="4">
         <v>3</v>
@@ -898,18 +941,18 @@
         <v>2</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="153" customHeight="1">
+    <row r="8" spans="1:26" ht="153" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C8" s="7">
         <v>3</v>
@@ -918,10 +961,10 @@
         <v>2</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>20</v>
+        <v>9</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>16</v>
       </c>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
@@ -944,12 +987,12 @@
       <c r="Y8" s="9"/>
       <c r="Z8" s="9"/>
     </row>
-    <row r="9" spans="1:26" ht="72">
+    <row r="9" spans="1:26" ht="84" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="4">
         <v>5</v>
@@ -958,10 +1001,10 @@
         <v>2</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>